<commit_message>
Highlight BSCR reconciliation matches and correct count formulas
</commit_message>
<xml_diff>
--- a/reporting/bscr/reconcile/results/BSCR_Reconciliation.xlsx
+++ b/reporting/bscr/reconcile/results/BSCR_Reconciliation.xlsx
@@ -11169,10 +11169,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0;[Red]\(#,##0\);0"/>
     <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\(#,##0.000\);0.000"/>
     <numFmt numFmtId="166" formatCode="[&gt;=0.0005]#,##0.000;[Red][&lt;=-0.0005]\(#,##0.000\);0.000"/>
+    <numFmt numFmtId="167" formatCode="&quot;MATCH&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;CHECK&quot;"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -11229,7 +11231,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -11266,6 +11268,36 @@
         <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -11279,7 +11311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -11379,13 +11411,70 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <numFmt numFmtId="167" formatCode="&quot;MATCH&quot;"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor indexed="64"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="&quot;CHECK&quot;"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor indexed="64"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -11423,11 +11512,11 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Legacy query: same pre-FX scale"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Required USD: same scale"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Required USD millions"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="USD">
-      <calculatedColumnFormula>E6*1.35</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Legacy USD / count">
+      <calculatedColumnFormula>IF([@Measure]="Count",[@[Legacy query: same pre-FX scale]],[@[Legacy query: same pre-FX scale]]*1.35)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{0B3803EC-9399-421A-86B9-0DEB9EBC8CA9}" name="Reconcile" dataDxfId="0">
-      <calculatedColumnFormula>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</calculatedColumnFormula>
+      <calculatedColumnFormula>IF([@Measure]="Count",[@[Legacy USD / count]]-[@[Template as saved]],[@[Legacy USD / count]]-[@[Required USD: same scale]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
@@ -12022,8 +12111,10 @@
       <c r="G5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="35" t="s">
-        <v>622</v>
+      <c r="H5" s="35" t="inlineStr">
+        <is>
+          <t>Legacy USD / count</t>
+        </is>
       </c>
       <c r="I5" t="s">
         <v>623</v>
@@ -12036,24 +12127,24 @@
       <c r="B6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="37">
         <v>5341</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="37">
         <v>5341</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="37">
         <v>5341</v>
       </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="24">
-        <f>E6*1.35</f>
-        <v>7210.35</v>
-      </c>
-      <c r="I6" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>7210.35</v>
+      <c r="F6" s="38"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="39">
+        <f>IF($B6="Count",$E6,$E6*1.35)</f>
+        <v>5341.0</v>
+      </c>
+      <c r="I6" s="41">
+        <f>IF($B6="Count",$H6-$C6,$H6-$F6)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12063,28 +12154,28 @@
       <c r="B7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="42">
         <v>29798684.509707961</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="42">
         <v>29798684.509707939</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="42">
         <v>29798684.509707939</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="43">
         <v>40228224.088105753</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="45">
         <v>40228.224088105737</v>
       </c>
-      <c r="H7" s="24">
-        <f t="shared" ref="H7:H20" si="0">E7*1.35</f>
-        <v>40228224.088105723</v>
-      </c>
-      <c r="I7" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>0</v>
+      <c r="H7" s="44">
+        <f>IF($B7="Count",$E7,$E7*1.35)</f>
+        <v>40228224.08810572</v>
+      </c>
+      <c r="I7" s="41">
+        <f>IF($B7="Count",$H7-$C7,$H7-$F7)</f>
+        <v>-2.9802322387695312e-08</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12094,28 +12185,28 @@
       <c r="B8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="46">
         <v>21558481.149128009</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="46">
         <v>21558481.14912812</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="46">
         <v>21558481.14912812</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="43">
         <v>29103949.55132281</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="45">
         <v>29103.94955132281</v>
       </c>
-      <c r="H8" s="24">
-        <f t="shared" si="0"/>
+      <c r="H8" s="44">
+        <f>IF($B8="Count",$E8,$E8*1.35)</f>
         <v>29103949.551322963</v>
       </c>
-      <c r="I8" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>1.5273690223693848E-7</v>
+      <c r="I8" s="41">
+        <f>IF($B8="Count",$H8-$C8,$H8-$F8)</f>
+        <v>1.5273690223693848e-07</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12125,24 +12216,24 @@
       <c r="B9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C9" s="47">
         <v>36</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="47">
         <v>36</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="47">
         <v>36</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="24">
-        <f t="shared" si="0"/>
-        <v>48.6</v>
-      </c>
-      <c r="I9" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>48.6</v>
+      <c r="F9" s="38"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="39">
+        <f>IF($B9="Count",$E9,$E9*1.35)</f>
+        <v>36.0</v>
+      </c>
+      <c r="I9" s="41">
+        <f>IF($B9="Count",$H9-$C9,$H9-$F9)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12152,28 +12243,28 @@
       <c r="B10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="46">
         <v>22066.496800000001</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="46">
         <v>22066.496800000001</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="46">
         <v>22066.496800000001</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="43">
         <v>29789.770680000001</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="45">
         <v>29.78977068</v>
       </c>
-      <c r="H10" s="24">
-        <f t="shared" si="0"/>
-        <v>29789.770680000001</v>
-      </c>
-      <c r="I10" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>0</v>
+      <c r="H10" s="44">
+        <f>IF($B10="Count",$E10,$E10*1.35)</f>
+        <v>29789.77068</v>
+      </c>
+      <c r="I10" s="41">
+        <f>IF($B10="Count",$H10-$C10,$H10-$F10)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12183,28 +12274,28 @@
       <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="42">
         <v>22066.496800000001</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="42">
         <v>22066.496800000001</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="42">
         <v>22066.496800000001</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="43">
         <v>29789.770680000001</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="45">
         <v>29.78977068</v>
       </c>
-      <c r="H11" s="24">
-        <f t="shared" si="0"/>
-        <v>29789.770680000001</v>
-      </c>
-      <c r="I11" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>0</v>
+      <c r="H11" s="44">
+        <f>IF($B11="Count",$E11,$E11*1.35)</f>
+        <v>29789.77068</v>
+      </c>
+      <c r="I11" s="41">
+        <f>IF($B11="Count",$H11-$C11,$H11-$F11)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12214,24 +12305,24 @@
       <c r="B12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="37">
         <v>173687</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="37">
         <v>173687</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="37">
         <v>173687</v>
       </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="24">
-        <f t="shared" si="0"/>
-        <v>234477.45</v>
-      </c>
-      <c r="I12" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>234477.45</v>
+      <c r="F12" s="38"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="39">
+        <f>IF($B12="Count",$E12,$E12*1.35)</f>
+        <v>173687.0</v>
+      </c>
+      <c r="I12" s="41">
+        <f>IF($B12="Count",$H12-$C12,$H12-$F12)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12241,28 +12332,28 @@
       <c r="B13" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="42">
         <v>121743087.30987801</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="42">
         <v>121743087.30988</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="42">
         <v>121743087.30988041</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="43">
         <v>164353167.86833531</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="45">
         <v>164353.16786833529</v>
       </c>
-      <c r="H13" s="24">
-        <f t="shared" si="0"/>
+      <c r="H13" s="44">
+        <f>IF($B13="Count",$E13,$E13*1.35)</f>
         <v>164353167.86833856</v>
       </c>
-      <c r="I13" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>3.2484531402587891E-6</v>
+      <c r="I13" s="41">
+        <f>IF($B13="Count",$H13-$C13,$H13-$F13)</f>
+        <v>3.248453140258789e-06</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12272,28 +12363,28 @@
       <c r="B14" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="46">
         <v>121743087.30987801</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="46">
         <v>121743087.30988</v>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="46">
         <v>121743087.30988041</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="43">
         <v>164353167.86833531</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="45">
         <v>164353.16786833529</v>
       </c>
-      <c r="H14" s="24">
-        <f t="shared" si="0"/>
+      <c r="H14" s="44">
+        <f>IF($B14="Count",$E14,$E14*1.35)</f>
         <v>164353167.86833856</v>
       </c>
-      <c r="I14" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>3.2484531402587891E-6</v>
+      <c r="I14" s="41">
+        <f>IF($B14="Count",$H14-$C14,$H14-$F14)</f>
+        <v>3.248453140258789e-06</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12303,24 +12394,24 @@
       <c r="B15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="47">
         <v>1970</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="47">
         <v>1970</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="47">
         <v>1970</v>
       </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="24">
-        <f t="shared" si="0"/>
-        <v>2659.5</v>
-      </c>
-      <c r="I15" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>2659.5</v>
+      <c r="F15" s="38"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="39">
+        <f>IF($B15="Count",$E15,$E15*1.35)</f>
+        <v>1970.0</v>
+      </c>
+      <c r="I15" s="41">
+        <f>IF($B15="Count",$H15-$C15,$H15-$F15)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12330,28 +12421,28 @@
       <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="46">
         <v>8046544.5189486863</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="46">
         <v>8046544.5189487049</v>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="46">
         <v>8046544.5189487059</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="43">
         <v>10862835.10058073</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="45">
         <v>10862.835100580731</v>
       </c>
-      <c r="H16" s="24">
-        <f t="shared" si="0"/>
+      <c r="H16" s="44">
+        <f>IF($B16="Count",$E16,$E16*1.35)</f>
         <v>10862835.100580754</v>
       </c>
-      <c r="I16" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>2.4214386940002441E-8</v>
+      <c r="I16" s="41">
+        <f>IF($B16="Count",$H16-$C16,$H16-$F16)</f>
+        <v>2.421438694000244e-08</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12361,28 +12452,28 @@
       <c r="B17" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="42">
         <v>6238734.9284093389</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="42">
         <v>6238734.9284093473</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="42">
         <v>6238734.9284093482</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F17" s="43">
         <v>8422292.153352607</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="45">
         <v>8422.2921533526078</v>
       </c>
-      <c r="H17" s="24">
-        <f t="shared" si="0"/>
-        <v>8422292.1533526201</v>
-      </c>
-      <c r="I17" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>0</v>
+      <c r="H17" s="44">
+        <f>IF($B17="Count",$E17,$E17*1.35)</f>
+        <v>8422292.15335262</v>
+      </c>
+      <c r="I17" s="41">
+        <f>IF($B17="Count",$H17-$C17,$H17-$F17)</f>
+        <v>1.30385160446167e-08</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12392,24 +12483,24 @@
       <c r="B18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="37">
         <v>90052</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="37">
         <v>90052</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="37">
         <v>90052</v>
       </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="24">
-        <f t="shared" si="0"/>
-        <v>121570.20000000001</v>
-      </c>
-      <c r="I18" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>121570.20000000001</v>
+      <c r="F18" s="38"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="39">
+        <f>IF($B18="Count",$E18,$E18*1.35)</f>
+        <v>90052.0</v>
+      </c>
+      <c r="I18" s="41">
+        <f>IF($B18="Count",$H18-$C18,$H18-$F18)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12419,28 +12510,28 @@
       <c r="B19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="42">
         <v>77561198.646257892</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="42">
         <v>77561198.646255136</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="42">
         <v>77561198.64625518</v>
       </c>
-      <c r="F19" s="13">
+      <c r="F19" s="43">
         <v>104707618.1724482</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="45">
         <v>104707.6181724482</v>
       </c>
-      <c r="H19" s="24">
-        <f t="shared" si="0"/>
+      <c r="H19" s="44">
+        <f>IF($B19="Count",$E19,$E19*1.35)</f>
         <v>104707618.17244451</v>
       </c>
-      <c r="I19" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>-3.6954879760742188E-6</v>
+      <c r="I19" s="41">
+        <f>IF($B19="Count",$H19-$C19,$H19-$F19)</f>
+        <v>-3.6954879760742188e-06</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.35">
@@ -12450,28 +12541,28 @@
       <c r="B20" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="46">
         <v>75864599.507855102</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="46">
         <v>75864599.50785242</v>
       </c>
-      <c r="E20" s="20">
+      <c r="E20" s="46">
         <v>75864599.507852465</v>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="43">
         <v>102417209.3356044</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="45">
         <v>102417.20933560441</v>
       </c>
-      <c r="H20" s="24">
-        <f t="shared" si="0"/>
+      <c r="H20" s="44">
+        <f>IF($B20="Count",$E20,$E20*1.35)</f>
         <v>102417209.33560084</v>
       </c>
-      <c r="I20" s="36">
-        <f>Recon102[[#This Row],[USD]]-Recon102[[#This Row],[Required USD: same scale]]</f>
-        <v>-3.5613775253295898E-6</v>
+      <c r="I20" s="41">
+        <f>IF($B20="Count",$H20-$C20,$H20-$F20)</f>
+        <v>-3.56137752532959e-06</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.35">
@@ -12487,8 +12578,10 @@
       <c r="H23" s="29"/>
     </row>
     <row r="24" spans="1:9" ht="41" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="31" t="s">
-        <v>53</v>
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>COLOUR KEY: yellow C–E = pre-FX template/output values; blue F/H = USD at the same scale; pale green G = USD millions. Reconcile: green MATCH / red CHECK. Green means agreement AFTER FX, not that the original template was already USD.</t>
+        </is>
       </c>
       <c r="B24" s="29"/>
       <c r="C24" s="29"/>
@@ -12523,8 +12616,10 @@
       <c r="H26" s="29"/>
     </row>
     <row r="27" spans="1:9" ht="41" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="31" t="s">
-        <v>56</v>
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>RECONCILE: count rows compare C, D and E exactly and never apply FX. Money rows compare H against F, and D against C after FX. Tolerance = 0.00001 in USD-thousand scale ($0.01). Numeric differences remain in I; MATCH/CHECK is only the display format.</t>
+        </is>
       </c>
       <c r="B27" s="29"/>
       <c r="C27" s="29"/>
@@ -26399,6 +26494,14 @@
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
   </mergeCells>
+  <conditionalFormatting sqref="I6:I20">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>IFERROR(AND(COUNT($C6:$E6)=3,IF($B6="Count",AND($C6=$D6,$D6=$E6,$I6=0),AND(ISNUMBER($F6),ISNUMBER($H6),ISNUMBER($I6),ABS($I6)&lt;=0.00001,ABS(($D6-$C6)*1.35)&lt;=0.00001))),FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
+      <formula>NOT(IFERROR(AND(COUNT($C6:$E6)=3,IF($B6="Count",AND($C6=$D6,$D6=$E6,$I6=0),AND(ISNUMBER($F6),ISNUMBER($H6),ISNUMBER($I6),ABS($I6)&lt;=0.00001,ABS(($D6-$C6)*1.35)&lt;=0.00001))),FALSE))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="B30" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
     <hyperlink ref="B31" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>

</xml_diff>